<commit_message>
Versão 1.8 já em produção
</commit_message>
<xml_diff>
--- a/dados/csv/registro_refugos.xlsx
+++ b/dados/csv/registro_refugos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G842"/>
+  <dimension ref="A1:G889"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24342,6 +24342,1369 @@
       <c r="F842" t="inlineStr"/>
       <c r="G842" t="inlineStr"/>
     </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>813623</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Batente alumínio (novo)</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>ACIONAMENTO</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>17/07/2026 15:43:12</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr"/>
+      <c r="G843" t="inlineStr"/>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>813521</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Borboleta</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>17/07/2026 15:43:35</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr"/>
+      <c r="G844" t="inlineStr"/>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>813271</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Carcaça BV3 inferior</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>17/07/2026 15:47:32</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr"/>
+      <c r="G845" t="inlineStr"/>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>813270</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Carcaça BV3 superior</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>17/07/2026 15:47:56</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr"/>
+      <c r="G846" t="inlineStr"/>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>813265</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Carcaça New BV superior</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>NEW BV</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>17/07/2026 15:49:04</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr"/>
+      <c r="G847" t="inlineStr"/>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>813310</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Cilindro da chave</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>17/07/2026 15:49:30</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr"/>
+      <c r="G848" t="inlineStr"/>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>813281</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Suporte orelha do BV</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>20/07/2026 07:00:23</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr"/>
+      <c r="G849" t="inlineStr"/>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>813053</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Acoplamento BV</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>23/07/2026 16:21:40</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr"/>
+      <c r="G850" t="inlineStr"/>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>813199</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Base de alumínio DZ</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:00:45</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr"/>
+      <c r="G851" t="inlineStr"/>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>813241</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Base Inferior Industrial</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:01:08</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr"/>
+      <c r="G852" t="inlineStr"/>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>813153</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Base superior Industrial</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:01:15</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr"/>
+      <c r="G853" t="inlineStr"/>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>813271</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Carcaça BV3 inferior</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:02:10</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr"/>
+      <c r="G854" t="inlineStr"/>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>813271</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Carcaça BV3 inferior</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:02:10</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr"/>
+      <c r="G855" t="inlineStr"/>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>813270</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Carcaça BV3 superior</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:02:30</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr"/>
+      <c r="G856" t="inlineStr"/>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>813259</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Carcaça New BV com encoder</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>NEW BV</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:02:52</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr"/>
+      <c r="G857" t="inlineStr"/>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>813525</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Eixo DZ novo</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>ENGRENAGEM</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:03:08</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr"/>
+      <c r="G858" t="inlineStr"/>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>813146</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Gomo alumínio</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>328</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>CREMALHEIRAS</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:03:38</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr"/>
+      <c r="G859" t="inlineStr"/>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>813281</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Suporte orelha do BV</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>24/07/2026 07:04:12</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr"/>
+      <c r="G860" t="inlineStr"/>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>813257</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Base da central NBV</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>NEW BV</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:08:37</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr"/>
+      <c r="G861" t="inlineStr"/>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>804246</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Base DZ superior Nylon</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:09:08</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr"/>
+      <c r="G862" t="inlineStr"/>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>813151</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Base DZ inferior Nylon</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:09:24</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr"/>
+      <c r="G863" t="inlineStr"/>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>804326</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Base Pivo New</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>PLACAS</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:09:49</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr"/>
+      <c r="G864" t="inlineStr"/>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>813260</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Calço estator NBV</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:10:42</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr"/>
+      <c r="G865" t="inlineStr"/>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>813080</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Gomo plástico</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>CREMALHEIRAS</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:11:10</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr"/>
+      <c r="G866" t="inlineStr"/>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>813317</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Mancal superior PV</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>ACIONAMENTO</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:11:55</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr"/>
+      <c r="G867" t="inlineStr"/>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>813316</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Porca fêmea</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>ACIONAMENTO</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:12:45</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr"/>
+      <c r="G868" t="inlineStr"/>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>813033</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Tampa da ventoinha</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:13:33</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr"/>
+      <c r="G869" t="inlineStr"/>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>813179</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Tampa do BV</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>BV</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:14:04</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr"/>
+      <c r="G870" t="inlineStr"/>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>804327</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Tampa Pivo New</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>PLACAS</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:14:37</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr"/>
+      <c r="G871" t="inlineStr"/>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>813248</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Tampa Grafite</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:15:02</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr"/>
+      <c r="G872" t="inlineStr"/>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>813024</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Tampa preta DZ</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:15:29</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr"/>
+      <c r="G873" t="inlineStr"/>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>813024</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Tampa preta DZ</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:15:29</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr"/>
+      <c r="G874" t="inlineStr"/>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>813025</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Ventoinha</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>MONTAGEM MOTOR</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:16:05</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr"/>
+      <c r="G875" t="inlineStr"/>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>804247</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Base da central DZ</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:16:35</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr"/>
+      <c r="G876" t="inlineStr"/>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>813525</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Eixo DZ novo</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:18:18</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr"/>
+      <c r="G877" t="inlineStr"/>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>813096</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Engrenagem ext DZ nova</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>ENGRENAGEM</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>24/07/2026 15:18:38</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr"/>
+      <c r="G878" t="inlineStr"/>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>813199</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Base de alumínio DZ</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:09:22</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr"/>
+      <c r="G879" t="inlineStr"/>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>813623</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Batente alumínio (novo)</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>ACIONAMENTO</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:10:32</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr"/>
+      <c r="G880" t="inlineStr"/>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>813521</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Borboleta</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>KIT</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:11:21</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr"/>
+      <c r="G881" t="inlineStr"/>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>813271</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Carcaça BV3 inferior</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:11:58</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr"/>
+      <c r="G882" t="inlineStr"/>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>813270</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Carcaça BV3 superior</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:12:17</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr"/>
+      <c r="G883" t="inlineStr"/>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>813311</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Chave PV alumínio</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>KIT</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:15:27</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr"/>
+      <c r="G884" t="inlineStr"/>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>813037</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Engrenagem DZ antiga</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>ENGRENAGEM</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:15:54</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr"/>
+      <c r="G885" t="inlineStr"/>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>813096</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Engrenagem ext DZ nova</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>ENGRENAGEM</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:16:12</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr"/>
+      <c r="G886" t="inlineStr"/>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>813146</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Gomo alumínio</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>CREMALHEIRAS</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:16:38</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr"/>
+      <c r="G887" t="inlineStr"/>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>813251</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Sem fim alumínio</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>MONTAGEM MOTOR</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:17:02</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr"/>
+      <c r="G888" t="inlineStr"/>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>813281</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Suporte orelha do BV</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>28/07/2026 16:17:29</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr"/>
+      <c r="G889" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>